<commit_message>
Group B: FS6402 SPEC (straight FSM x JIC swivel, nose from the record CC), closed loop 0 off
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/stage/orfs_tables/DesignTable_FS6402.xlsx
+++ b/tools/_out/groupB_20261021/stage/orfs_tables/DesignTable_FS6402.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,90 +426,95 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
+          <t>SNT@DRIVE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>$PRP@PartNo</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>$PRP@Description</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>$PRP@DataStatus</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>$PRP@AxialSource</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>$COMMENT</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>$PRP@ScopeAction</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>$PRP@OMiSKU</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>$PRP@OnWebsite</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>$PRP@DimSource</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>L@DRIVE</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>S1HEX@HEX</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>SHEX@HEX</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>THDMAJ_D@DRIVE</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>THDMAJ_B@DRIVE</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>$PRP@Thread_D</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>$PRP@Thread_B</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>$PRP@TubeOD</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>D1@BORE</t>
         </is>
@@ -521,80 +526,86 @@
           <t>FS6402-04-04</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" t="n">
+        <v>0.355</v>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>FS6402-04-04</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>04 MFS - 04 FJS Straight</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "L LGTH" = "1.344" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 448.4, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "H HEX" = "0.625" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 448.4, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "C HEX" = "0.562" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 448.4, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -04 = 0.5625 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "A THREAD" "9/16-18" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -04 = 0.4375 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "B THREAD" "7/16-20" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "A THREAD" "9/16-18" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "B THREAD" "7/16-20" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "TUBE O.D." "1/4" in the table's format</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5556 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-04-04 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: D1@BORE, SNT@DRIVE] [BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "L LGTH" = "1.344" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 448.4, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "H HEX" = "0.625" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 448.4, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "C HEX" = "0.562" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 448.4, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -04 = 0.5625 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "A THREAD" "9/16-18" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -04 = 0.4375 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "B THREAD" "7/16-20" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "A THREAD" "9/16-18" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "B THREAD" "7/16-20" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-04-04 col "TUBE O.D." "1/4" in the table's format</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5556 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-04-04 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6402-04-04 (PARTcommunity / CADENAS, group B 2026-10-21: D1@BORE=AD, SNT@DRIVE=CC; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>FS6402-04-04</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>yes - OMi website ORFS list (two passes, omi_skus_orfs.txt)</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>1.344</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>0.625</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>0.5620000000000001</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>0.5625</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>0.4375</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>9/16-18</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>7/16-20</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>1/4</t>
         </is>
+      </c>
+      <c r="T3" t="n">
+        <v>0.172</v>
       </c>
     </row>
     <row r="4">
@@ -603,82 +614,85 @@
           <t>FS6402-06-06</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>FS6402-06-06</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>06 MFS - 06 FJS Straight</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "L LGTH" = "1.565" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 458.4, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "H HEX" = "0.750" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 458.4, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "C HEX" = "0.688" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 458.4, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -06 = 0.6875 (PLAN.md s2 FS_THR / the -06 thread of every staged ORFS row); = Brennan "A THREAD" "11/16-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -06 = 0.5625 (PLAN.md s2 FS_THR / the -06 thread of every staged ORFS row); = Brennan "B THREAD" "9/16-18" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "A THREAD" "11/16-16" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "B THREAD" "9/16-18" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "TUBE O.D." "3/8" in the table's format; D1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: straight ORFS tables: FSM -06 bore on 28 Air-Way row(s) in 8 tables: 0.26 x28 (unanimous) [Air-Way, not Brennan]</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5557 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-06-06 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: SNT@DRIVE] [BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "L LGTH" = "1.565" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 458.4, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "H HEX" = "0.750" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 458.4, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "C HEX" = "0.688" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 458.4, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -06 = 0.6875 (PLAN.md s2 FS_THR / the -06 thread of every staged ORFS row); = Brennan "A THREAD" "11/16-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -06 = 0.5625 (PLAN.md s2 FS_THR / the -06 thread of every staged ORFS row); = Brennan "B THREAD" "9/16-18" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "A THREAD" "11/16-16" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "B THREAD" "9/16-18" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-06-06 col "TUBE O.D." "3/8" in the table's format; D1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: straight ORFS tables: FSM -06 bore on 28 Air-Way row(s) in 8 tables: 0.26 x28 (unanimous) [Air-Way, not Brennan]</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5557 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-06-06 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6402-06-06 (PARTcommunity / CADENAS, group B 2026-10-21: SNT@DRIVE=CC; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>FS6402-06-06</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>yes - OMi website ORFS list (two passes, omi_skus_orfs.txt)</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>1.565</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>0.75</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>0.6879999999999999</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>0.6875</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>0.5625</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>11/16-16</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>9/16-18</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>3/8</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>0.26</v>
       </c>
     </row>
@@ -688,80 +702,86 @@
           <t>FS6402-08-08</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" t="n">
+        <v>0.422</v>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>FS6402-08-08</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>08 MFS - 08 FJS Straight</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "L LGTH" = "1.770" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 468.5, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "H HEX" = "0.875" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 468.5, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "C HEX" = "0.875" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 468.5, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -08 = 0.8125 (PLAN.md s2 FS_THR / the -08 thread of every staged ORFS row); = Brennan "A THREAD" "13/16-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -08 = 0.75 (PLAN.md s2 FS_THR / the -08 thread of every staged ORFS row); = Brennan "B THREAD" "3/4-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "A THREAD" "13/16-16" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "B THREAD" "3/4-16" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "TUBE O.D." "1/2" in the table's format</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5558 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-08-08 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: D1@BORE, SNT@DRIVE] [BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "L LGTH" = "1.770" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 468.5, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "H HEX" = "0.875" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 468.5, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "C HEX" = "0.875" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 468.5, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -08 = 0.8125 (PLAN.md s2 FS_THR / the -08 thread of every staged ORFS row); = Brennan "A THREAD" "13/16-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -08 = 0.75 (PLAN.md s2 FS_THR / the -08 thread of every staged ORFS row); = Brennan "B THREAD" "3/4-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "A THREAD" "13/16-16" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "B THREAD" "3/4-16" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-08-08 col "TUBE O.D." "1/2" in the table's format</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5558 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-08-08 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6402-08-08 (PARTcommunity / CADENAS, group B 2026-10-21: D1@BORE=AD, SNT@DRIVE=CC; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>FS6402-08-08</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>yes - OMi website ORFS list (two passes, omi_skus_orfs.txt)</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>1.77</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.875</v>
       </c>
       <c r="M5" t="n">
         <v>0.875</v>
       </c>
       <c r="N5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="O5" t="n">
         <v>0.8125</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>0.75</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>13/16-16</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>3/4-16</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
+      </c>
+      <c r="T5" t="n">
+        <v>0.378</v>
       </c>
     </row>
     <row r="6">
@@ -770,80 +790,86 @@
           <t>FS6402-10-10</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>FS6402-10-10</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>10 MFS - 10 FJS Straight</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "L LGTH" = "2.060" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 478.6, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "H HEX" = "1.062" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 478.6, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "C HEX" = "1.000" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 478.6, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -10 = 1.0 (PLAN.md s2 FS_THR / the -10 thread of every staged ORFS row); = Brennan "A THREAD" "1-14" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -10 = 0.875 (PLAN.md s2 FS_THR / the -10 thread of every staged ORFS row); = Brennan "B THREAD" "7/8-14" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "A THREAD" "1-14" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "B THREAD" "7/8-14" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "TUBE O.D." "5/8" in the table's format</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5559 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-10-10 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: D1@BORE, SNT@DRIVE] [BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "L LGTH" = "2.060" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 478.6, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "H HEX" = "1.062" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 478.6, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "C HEX" = "1.000" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 478.6, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -10 = 1.0 (PLAN.md s2 FS_THR / the -10 thread of every staged ORFS row); = Brennan "A THREAD" "1-14" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -10 = 0.875 (PLAN.md s2 FS_THR / the -10 thread of every staged ORFS row); = Brennan "B THREAD" "7/8-14" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "A THREAD" "1-14" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "B THREAD" "7/8-14" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-10-10 col "TUBE O.D." "5/8" in the table's format</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5559 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-10-10 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6402-10-10 (PARTcommunity / CADENAS, group B 2026-10-21: D1@BORE=AD, SNT@DRIVE=CC; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>FS6402-10-10</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>yes - OMi website ORFS list (two passes, omi_skus_orfs.txt)</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>2.06</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>1.062</v>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
       </c>
       <c r="O6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
         <v>0.875</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1-14</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>7/8-14</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>5/8</t>
         </is>
+      </c>
+      <c r="T6" t="n">
+        <v>0.484</v>
       </c>
     </row>
     <row r="7">
@@ -852,82 +878,85 @@
           <t>FS6402-12-12</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>FS6402-12-12</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>12 MFS - 12 FJS Straight</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: L@DRIVE] [BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "H HEX" = "1.250" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 488.7, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "C HEX" = "1.250" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 488.7, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -12 = 1.1875 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "A THREAD" "1 3/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -12 = 1.0625 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "B THREAD" "1 1/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "A THREAD" "1 3/16-12" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "B THREAD" "1 1/16-12" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "TUBE O.D." "3/4" in the table's format; D1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: straight ORFS tables: FSM -12 bore on 24 Air-Way row(s) in 8 tables: 0.61 x24 (unanimous) [Air-Way, not Brennan]</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5560 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-12-12 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6402-12-12 (PARTcommunity / CADENAS, L@DRIVE=L; user 2026-10-21 "yes you can use them following my rule")</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: SNT@DRIVE] [BRENNAN-CAD 2026-10-21: L@DRIVE] [BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "H HEX" = "1.250" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 488.7, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "C HEX" = "1.250" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 488.7, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -12 = 1.1875 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "A THREAD" "1 3/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -12 = 1.0625 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "B THREAD" "1 1/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "A THREAD" "1 3/16-12" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "B THREAD" "1 1/16-12" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-12-12 col "TUBE O.D." "3/4" in the table's format; D1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: straight ORFS tables: FSM -12 bore on 24 Air-Way row(s) in 8 tables: 0.61 x24 (unanimous) [Air-Way, not Brennan]</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5560 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-12-12 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6402-12-12 (PARTcommunity / CADENAS, L@DRIVE=L; user 2026-10-21 "yes you can use them following my rule") | Brennan CAD record FS6402-12-12 (PARTcommunity / CADENAS, group B 2026-10-21: SNT@DRIVE=CC; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>FS6402-12-12</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>yes - OMi website ORFS list (two passes, omi_skus_orfs.txt)</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>2.25</v>
-      </c>
-      <c r="L7" t="n">
-        <v>1.25</v>
       </c>
       <c r="M7" t="n">
         <v>1.25</v>
       </c>
       <c r="N7" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="O7" t="n">
         <v>1.1875</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>1.0625</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>1 3/16-12</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>1 1/16-12</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>3/4</t>
         </is>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>0.61</v>
       </c>
     </row>
@@ -937,82 +966,85 @@
           <t>FS6402-16-16</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>FS6402-16-16</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>16 MFS - 16 FJS Straight</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "L LGTH" = "2.460" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 498.8, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "H HEX" = "1.500" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 498.8, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "C HEX" = "1.500" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 498.8, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -16 = 1.4375 (PLAN.md s2 FS_THR / the -16 thread of every staged ORFS row); = Brennan "A THREAD" "1 7/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -16 = 1.3125 (PLAN.md s2 FS_THR / the -16 thread of every staged ORFS row); = Brennan "B THREAD" "1 5/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "A THREAD" "1 7/16-12" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "B THREAD" "1 5/16-12" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "TUBE O.D." "1" in the table's format; D1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: straight ORFS tables: FSM -16 bore on 25 Air-Way row(s) in 8 tables: 0.81 x25 (unanimous) [Air-Way, not Brennan]</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5561 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-16-16 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: SNT@DRIVE] [BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "L LGTH" = "2.460" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 498.8, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "H HEX" = "1.500" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 498.8, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "C HEX" = "1.500" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 498.8, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -16 = 1.4375 (PLAN.md s2 FS_THR / the -16 thread of every staged ORFS row); = Brennan "A THREAD" "1 7/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -16 = 1.3125 (PLAN.md s2 FS_THR / the -16 thread of every staged ORFS row); = Brennan "B THREAD" "1 5/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "A THREAD" "1 7/16-12" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "B THREAD" "1 5/16-12" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-16-16 col "TUBE O.D." "1" in the table's format; D1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: straight ORFS tables: FSM -16 bore on 25 Air-Way row(s) in 8 tables: 0.81 x25 (unanimous) [Air-Way, not Brennan]</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5561 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-16-16 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6402-16-16 (PARTcommunity / CADENAS, group B 2026-10-21: SNT@DRIVE=CC; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>FS6402-16-16</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>yes - OMi website ORFS list (two passes, omi_skus_orfs.txt)</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>2.46</v>
-      </c>
-      <c r="L8" t="n">
-        <v>1.5</v>
       </c>
       <c r="M8" t="n">
         <v>1.5</v>
       </c>
       <c r="N8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="O8" t="n">
         <v>1.4375</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>1.3125</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>1 7/16-12</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>1 5/16-12</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>0.8100000000000001</v>
       </c>
     </row>
@@ -1022,82 +1054,85 @@
           <t>FS6402-20-20</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>FS6402-20-20</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>20 MFS - 20 FJS Straight</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "L LGTH" = "2.615" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 508.8, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "H HEX" = "1.750" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 508.8, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "C HEX" = "2.000" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 508.8, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -20 = 1.6875 (PLAN.md s2 FS_THR / the -20 thread of every staged ORFS row); = Brennan "A THREAD" "1-11/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -20 = 1.625 (PLAN.md s2 FS_THR / the -20 thread of every staged ORFS row); = Brennan "B THREAD" "1-5/8-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "A THREAD" "1-11/16-12" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "B THREAD" "1-5/8-12" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "TUBE O.D." "1 1/4" in the table's format; D1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: straight ORFS tables: FSM -20 bore on 16 Air-Way row(s) in 8 tables: 1.02 x16 (unanimous) [Air-Way, not Brennan]</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5562 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-20-20 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: SNT@DRIVE] [BRENNAN-ONLY 2026-10-18] no Air-Way row -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L@DRIVE: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "L LGTH" = "2.615" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 508.8, page verified True) [Brennan = yes 2026-10-18] - FS face -&gt; JIC swivel nut face (overall); mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); S1HEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "H HEX" = "1.750" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 508.8, page verified True) [Brennan = yes 2026-10-18] - body hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); SHEX@HEX: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "C HEX" = "2.000" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 508.8, page verified True) [Brennan = yes 2026-10-18] - JIC swivel nut hex; mapping: no row of this table has both an Air-Way and a Brennan value (drawing mapping only; cross-check in evidence/crosscheck.txt); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -20 = 1.6875 (PLAN.md s2 FS_THR / the -20 thread of every staged ORFS row); = Brennan "A THREAD" "1-11/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_B@DRIVE: end library: straight (UN/UNF) thread of dash -20 = 1.625 (PLAN.md s2 FS_THR / the -20 thread of every staged ORFS row); = Brennan "B THREAD" "1-5/8-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "A THREAD" "1-11/16-12" in the table's format; $PRP@Thread_B: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "B THREAD" "1-5/8-12" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p5 table ORFS-p005-t04 "FS6402 MFS-FJS STRAIGHT" row FS6402-20-20 col "TUBE O.D." "1 1/4" in the table's format; D1@BORE: per-dash transfer, user 2026-10-18 Q-FS-XFER yes: straight ORFS tables: FSM -20 bore on 16 Air-Way row(s) in 8 tables: 1.02 x16 (unanimous) [Air-Way, not Brennan]</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) (Brennan prints it: Brennan-only stays MISSING) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5562 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p5 FS6402-20-20 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6402-20-20 (PARTcommunity / CADENAS, group B 2026-10-21: SNT@DRIVE=CC; user 2026-10-21 "yes you can use them following my rule")</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>FS6402-20-20</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>yes - OMi website ORFS list (two passes, omi_skus_orfs.txt)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>2.615</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>1.75</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>2</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>1.6875</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>1.625</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>1 11/16-12</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>1 5/8-12</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>1 1/4</t>
         </is>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>1.02</v>
       </c>
     </row>
@@ -1107,37 +1142,37 @@
           <t>FS6402-24-24</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>FS6402-24-24</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>24 MFS - 24 FJS Straight</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>no Air-Way row</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>DROP: in OMi's parts file but NOT on OMi's website (OMi website ORFS list (two passes, omi_skus_orfs.txt)) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | no Air-Way MFS x female JIC swivel series (Air-Way FF6402 is MORB x FFSS = OMi FS6540; Brennan FS6402 only) | OMi parts file row 5563 (no dimensions)</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>no - OMi website ORFS list (two passes, omi_skus_orfs.txt)</t>
         </is>

</xml_diff>